<commit_message>
VP scoreboard: cooldown is a per-item timeout that raises UVM_FATAL
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DzTYgXHQRdW29cqRnE8XYg
</commit_message>
<xml_diff>
--- a/Control_Stage_VP.xlsx
+++ b/Control_Stage_VP.xlsx
@@ -715,12 +715,12 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Cycle-by-cycle compare of monitor vs model. Two check families: DATA checks and TIMING checks; timing checks have a COOLDOWN (see sheet 'Scoreboard').</t>
+          <t>Compares expected items (from the model) with DUT items (from the monitor), by channel. Every expected item has a COOLDOWN counter: no matching DUT item after N cycles -&gt; UVM_FATAL (see sheet 'Scoreboard').</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Not queue-based: CTRL has no bubble, so expected cycle k must match observed cycle k.</t>
+          <t>CTRL has no bubble and fixed latency, so the n-th expected item must be matched by the n-th DUT item at the predicted cycle.</t>
         </is>
       </c>
     </row>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1012,14 +1012,14 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>VP — Scoreboard: data checks, timing checks and cooldown</t>
+          <t>VP — Scoreboard: data checks, timing checks and cooldown (timeout)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="44" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>CTRL has no bubble and fixed latency, so the scoreboard compares cycle k observed against cycle k expected (not a queue). Timing checks (SB-T*) have a cooldown so one slipped cycle does not flood the log; the first error is always reported.</t>
+          <t>Every expected item sent by the reference model starts a cooldown counter (counted in clock cycles). If the matching DUT item has not arrived when it expires, the scoreboard raises UVM_FATAL. Data checks (SB-D*) compare content, timing checks (SB-T*) compare arrival cycle.</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1078,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>All 16 LRs observed through the bind probe == model, after every cycle.</t>
+          <t>Matching DUT item (16 LRs from the bind probe, per cycle) == expected item from the model.</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -1093,11 +1093,11 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Not blanked by timing cooldown. Blanked only in RESET cooldown (LR reset value not specified, Q6).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="47" customHeight="1">
+          <t>Expected item starts a cooldown counter; no DUT item before it expires -&gt; UVM_FATAL (rule C2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
           <t>SB-D02</t>
@@ -1115,12 +1115,12 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>mult / acc / aaq / str bus == model (slot fields + resolved post-LR-write operand values).</t>
+          <t>mult / acc / aaq / str bus == expected (slot fields + resolved post-LR-write operand values).</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>Every cycle that the model says a word executes.</t>
+          <t>Every cycle the model says a word executes.</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
@@ -1130,7 +1130,7 @@
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Reported normally. If a timing violation was reported, mismatches during its cooldown are only counted (see rule C4).</t>
+          <t>Same cooldown / FATAL rule.</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1152,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>xmem_read_en and (when en = 1) xmem_read_addr == model.</t>
+          <t>xmem_read_en and (when en = 1) xmem_read_addr == expected.</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Same as SB-D02.</t>
+          <t>Same cooldown / FATAL rule.</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Executed PC / inst$ word (probe) == model PC / word.</t>
+          <t>Executed PC / inst$ word (probe) == expected PC / word.</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -1204,7 +1204,7 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Same as SB-D02.</t>
+          <t>Same cooldown / FATAL rule.</t>
         </is>
       </c>
     </row>
@@ -1226,12 +1226,12 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>After the HALT word: PC and inst$ hold, buses carry no new word, xmem_read_en = 0, LR file unchanged.</t>
+          <t>After the HALT word: PC and inst$ hold, no new bus word, xmem_read_en = 0, LR file unchanged.</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>From the cycle after HALT until restart or reset.</t>
+          <t>From the cycle after HALT until restart / reset.</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
@@ -1241,11 +1241,11 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Not blanked (this is the check that cooldown must never hide).</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="34" customHeight="1">
+          <t>No expected item exists, so no cooldown: any DUT activity is an unexpected item -&gt; UVM_ERROR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="47" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
           <t>SB-T01</t>
@@ -1258,17 +1258,17 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>No bubble / no skip</t>
+          <t>Arrival cycle (exact)</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Observed cycle k carries exactly the word the model expects for cycle k: one word per cycle, none missing, none repeated.</t>
+          <t>The matching DUT item arrives exactly at the cycle the model predicts (fixed latency, no bubble).</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Every cycle from first dispatch until HALT.</t>
+          <t>Every item.</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
@@ -1278,11 +1278,11 @@
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Report first violation, then cooldown (rules C1-C3).</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="34" customHeight="1">
+          <t>Item arrives inside the cooldown but at the wrong cycle -&gt; UVM_ERROR (timing), compare still done. Never arrives -&gt; FATAL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="47" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>SB-T02</t>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>First dispatch comes exactly START_LATENCY cycles after the start event.</t>
+          <t>First DUT item arrives exactly START_LATENCY cycles after the start event.</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -1315,7 +1315,7 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>START_LATENCY is a parameter – value and start event are Spec Question Q13.</t>
+          <t>START_LATENCY is a parameter – value and start event are Spec Question Q13. The cooldown of the first item must be &gt;= START_LATENCY.</t>
         </is>
       </c>
     </row>
@@ -1337,7 +1337,7 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>The word after a branch (taken or not) executes in the very next cycle; the non-chosen candidate never executes.</t>
+          <t>The word after a branch (taken or not) arrives the very next cycle; the non-chosen candidate never produces an item.</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Same as SB-T01.</t>
+          <t>Missing item -&gt; FATAL (C2); item of the non-chosen candidate -&gt; unexpected item, UVM_ERROR (C3).</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>An LR write of word N is visible to the lanes / branch of word N+1, never in word N; buses see it in word N.</t>
+          <t>An LR write of word N shows in the LR item of the cycle after N, and in the bus items of word N.</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -1389,11 +1389,11 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Same as SB-T01.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="34" customHeight="1">
+          <t>Wrong cycle -&gt; UVM_ERROR (timing).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="47" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
           <t>SB-T05</t>
@@ -1411,7 +1411,7 @@
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>While rst = 1 nothing is dispatched; after rst release PC = 0 and the first word follows with START_LATENCY.</t>
+          <t>On rst the expected queue and all cooldown counters are flushed; after release PC = 0 and the first item arrives after START_LATENCY.</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
@@ -1426,11 +1426,11 @@
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>RESET cooldown (rule C5) applies first, then normal timing checks resume.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="34" customHeight="1">
+          <t>No cooldown runs while rst = 1; first item's cooldown starts at rst release (rule C6).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
           <t>SB-T06</t>
@@ -1443,63 +1443,83 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
+          <t>Unexpected DUT item</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>A DUT item arrives and no expected item is pending.</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Every DUT item.</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>UVM_ERROR (rule C3).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>SB-T07</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>TIMING</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
           <t>Memory-wait timing (placeholder)</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Stall behavior of PC, LR commit, buses and load port.</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Stall behavior of PC, LR commit, buses and load port; cooldown must be paused / extended while the DUT legally waits.</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F16" s="7" t="inlineStr">
         <is>
           <t>MEM-01</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>DISABLED until the memory-wait spec is released.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>Timing cooldown — rules</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="9" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>Purpose: one slipped cycle shifts every later cycle, so without a cooldown a single timing bug produces hundreds of follow-on errors. The cooldown keeps the log readable but never hides the first error.</t>
-        </is>
-      </c>
-      <c r="C18" s="10" t="n"/>
-      <c r="D18" s="10" t="n"/>
-      <c r="E18" s="10" t="n"/>
-      <c r="F18" s="10" t="n"/>
-      <c r="G18" s="10" t="n"/>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>DISABLED until the memory-wait spec is released (rule C7).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Cooldown (timeout) — rules</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>State machine per timing check: ARMED → (violation) → REPORTED → COOLDOWN(N cycles) → ARMED. In ARMED the checker reports every violation. The FIRST violation is always reported as UVM_ERROR with cycle number, expected and observed record.</t>
+          <t>Meaning: the cooldown is the maximum number of clock cycles the scoreboard waits for the DUT item that belongs to an expected (reference) item. It is a watchdog, not a tolerance for late data.</t>
         </is>
       </c>
       <c r="C19" s="10" t="n"/>
@@ -1508,15 +1528,15 @@
       <c r="F19" s="10" t="n"/>
       <c r="G19" s="10" t="n"/>
     </row>
-    <row r="20" ht="34" customHeight="1">
+    <row r="20" ht="47" customHeight="1">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>COOLDOWN: further timing violations of the same check (and its family SB-T*) are counted in 'suppressed_timing_errors' and NOT reported. The counter restarts at N on each suppressed violation, so a continuous slip ends one cooldown after it stops. After the cooldown the check re-arms; a violation after that is reported again.</t>
+          <t>Mechanism: when the reference model delivers an expected item to the scoreboard it is stored with a counter that is incremented every clock cycle (the 'time steps'). When the matching DUT item arrives, it is compared and the expected item is removed. If the counter passes COOLDOWN_CYCLES and no DUT item has arrived -&gt; UVM_FATAL 'SB_TIMEOUT' with the expected item (cycle, PC, word, bus values) printed. FATAL because nothing can be compared any more and every later item would be wrong too.</t>
         </is>
       </c>
       <c r="C20" s="10" t="n"/>
@@ -1528,12 +1548,12 @@
     <row r="21" ht="34" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>Data checks (SB-D01..D04) are never switched off by the timing cooldown. During a cooldown their mismatches are COUNTED but not printed one by one (knob DATA_IN_COOLDOWN = COUNT_ONLY, default) or printed normally (= REPORT). SB-D05 is always reported.</t>
+          <t>Opposite direction: a DUT item that arrives while no expected item is pending -&gt; UVM_ERROR 'unexpected item' (not FATAL – the expected stream is still intact). Arrival at a wrong cycle inside the cooldown -&gt; UVM_ERROR (SB-T01), the data compare is still done.</t>
         </is>
       </c>
       <c r="C21" s="10" t="n"/>
@@ -1545,12 +1565,12 @@
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>C5</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>RESET cooldown: for RESET_COOLDOWN_CYCLES after rst release, SB-D01 and SB-T01..T04 are blanked (LR reset value and exact restart behavior are not specified – Q6, Q13). SB-T05 is the only timing check active in that window.</t>
+          <t>Separate counter per channel (LR probe, 4 buses, xmem port, PC trace), so the FATAL message names the channel that stopped. Default COOLDOWN_CYCLES is the same for all and can be overridden per channel.</t>
         </is>
       </c>
       <c r="C22" s="10" t="n"/>
@@ -1562,12 +1582,12 @@
     <row r="23" ht="34" customHeight="1">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>C6</t>
+          <t>C5</t>
         </is>
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>Resync option (RESYNC_AFTER_COOLDOWN = 1): when the cooldown ends, the model pointer is re-aligned to the observed PC so the rest of the kernel can still be compared. If 0, the kernel is marked failed and the compare stops at the end of the cooldown.</t>
+          <t>End of test: in check_phase every expected queue must be empty. Items still pending after the last cycle -&gt; UVM_FATAL 'SB_PENDING'. The test also waits at least COOLDOWN_CYCLES after the HALT word retires before ending, so late items are not missed.</t>
         </is>
       </c>
       <c r="C23" s="10" t="n"/>
@@ -1579,12 +1599,12 @@
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>C7</t>
+          <t>C6</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>Cooldown never crosses a kernel boundary: at kernel start (or reset) all checks re-arm, the cooldown counters are cleared.</t>
+          <t>Reset: rst flushes all expected queues and clears all counters. No counter runs while rst = 1. The first expected item after reset starts its counter at rst release (so START_LATENCY must fit inside the cooldown).</t>
         </is>
       </c>
       <c r="C24" s="10" t="n"/>
@@ -1596,12 +1616,12 @@
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>C8</t>
+          <t>C7</t>
         </is>
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>Pass / fail: the test FAILS if the number of reported errors is &gt; 0 OR 'suppressed_timing_errors' &gt; 0. The suppressed count is printed in the final report so cooldown can never produce a silent pass.</t>
+          <t>Memory wait (MEM-01): the spec does not define it yet. When it does, the counter must be paused (or the cooldown extended) while the DUT legally stalls; until then a stall looks like a timeout. The check is disabled.</t>
         </is>
       </c>
       <c r="C25" s="10" t="n"/>
@@ -1613,12 +1633,12 @@
     <row r="26" ht="22" customHeight="1">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>C9</t>
+          <t>C8</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>Parameters: COOLDOWN_CYCLES (default 4), RESET_COOLDOWN_CYCLES (default 2), DATA_IN_COOLDOWN (COUNT_ONLY | REPORT), RESYNC_AFTER_COOLDOWN (0|1), START_LATENCY (spec TBD). Defaults are starting values to tune after the first runs.</t>
+          <t>Value: since CTRL has fixed latency, COOLDOWN_CYCLES can be small (starting value 16 cycles, must be &gt;= START_LATENCY + 1). A large value only delays the FATAL; exact timing is checked by SB-T01, not by the cooldown.</t>
         </is>
       </c>
       <c r="C26" s="10" t="n"/>
@@ -1626,6 +1646,23 @@
       <c r="E26" s="10" t="n"/>
       <c r="F26" s="10" t="n"/>
       <c r="G26" s="10" t="n"/>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>Parameters: COOLDOWN_CYCLES (default 16), COOLDOWN_&lt;channel&gt; overrides, START_LATENCY (spec TBD), STOP_ON_FATAL (UVM default). The max observed arrival delay per channel is printed in the final report to help tune the value.</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="n"/>
+      <c r="D27" s="10" t="n"/>
+      <c r="E27" s="10" t="n"/>
+      <c r="F27" s="10" t="n"/>
+      <c r="G27" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -1633,12 +1670,12 @@
     <mergeCell ref="B19:G19"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A18:G18"/>
     <mergeCell ref="B22:G22"/>
     <mergeCell ref="B23:G23"/>
+    <mergeCell ref="B27:G27"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="B26:G26"/>
-    <mergeCell ref="B18:G18"/>
     <mergeCell ref="B21:G21"/>
     <mergeCell ref="B25:G25"/>
   </mergeCells>
@@ -4689,15 +4726,15 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="34" customHeight="1">
+    <row r="17" ht="47" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>cg_timing_cooldown</t>
+          <t>cg_arrival_delay</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Cooldown entered (per check), suppressed count &gt; 0, resync used – expected EMPTY in a passing regression; used to prove the checker was exercised in negative tests.</t>
+          <t>Cycles between expected item and matching DUT item, per channel (0 .. COOLDOWN_CYCLES) – should hit only the exact-latency bin; used to tune COOLDOWN_CYCLES. Negative test: cooldown FATAL and unexpected-item ERROR each fired at least once.</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">

</xml_diff>